<commit_message>
preserve max batch size test logs
</commit_message>
<xml_diff>
--- a/finetune/toolkit/toolkit_v2.3.1_python312/Log/Max_batchsize_gemma-3-12b-it_2026-09-10_095521/performance_result_2026-09-10_095534.xlsx
+++ b/finetune/toolkit/toolkit_v2.3.1_python312/Log/Max_batchsize_gemma-3-12b-it_2026-09-10_095521/performance_result_2026-09-10_095534.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="ENV Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Performance Info" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,4 +564,1932 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Test Model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GPU Used Num</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Seq_len</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Gradient_accumulation_steps</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gemma-3-12b-it</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[Dataset(dataset_path='../../products/aiDAPTIVLink/toolkit_dataset_10k.json', strategy='qa', image_folder='', images_per_row=1)]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Batch size</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1st Efficiency(token/s)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2nd Efficiency(token/s)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3rd Efficiency(token/s)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Avg Efficiency(2~3)(token/s)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10M Dataset training time</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
+        <v>107.11</v>
+      </c>
+      <c r="C4" t="n">
+        <v>115.34</v>
+      </c>
+      <c r="D4" t="n">
+        <v>115.37</v>
+      </c>
+      <c r="E4" t="n">
+        <v>115.355</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>86688.92 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>208.59</v>
+      </c>
+      <c r="C5" t="n">
+        <v>224.45</v>
+      </c>
+      <c r="D5" t="n">
+        <v>224.15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>224.3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>44583.15 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="n">
+        <v>308.06</v>
+      </c>
+      <c r="C6" t="n">
+        <v>332.46</v>
+      </c>
+      <c r="D6" t="n">
+        <v>333.3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>332.88</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>30040.86 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="n">
+        <v>401.88</v>
+      </c>
+      <c r="C7" t="n">
+        <v>426.57</v>
+      </c>
+      <c r="D7" t="n">
+        <v>427.42</v>
+      </c>
+      <c r="E7" t="n">
+        <v>426.995</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>23419.48 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>477.86</v>
+      </c>
+      <c r="C8" t="n">
+        <v>512.29</v>
+      </c>
+      <c r="D8" t="n">
+        <v>513.02</v>
+      </c>
+      <c r="E8" t="n">
+        <v>512.655</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>19506.3 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="n">
+        <v>554.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>593.42</v>
+      </c>
+      <c r="D9" t="n">
+        <v>592.25</v>
+      </c>
+      <c r="E9" t="n">
+        <v>592.835</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>16868.1 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="n">
+        <v>623.58</v>
+      </c>
+      <c r="C10" t="n">
+        <v>667.52</v>
+      </c>
+      <c r="D10" t="n">
+        <v>668.83</v>
+      </c>
+      <c r="E10" t="n">
+        <v>668.175</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>14966.14 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="n">
+        <v>693.8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>738.95</v>
+      </c>
+      <c r="D11" t="n">
+        <v>743.63</v>
+      </c>
+      <c r="E11" t="n">
+        <v>741.29</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>13490.0 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="n">
+        <v>767.51</v>
+      </c>
+      <c r="C12" t="n">
+        <v>803.25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>804</v>
+      </c>
+      <c r="E12" t="n">
+        <v>803.625</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>12443.61 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" t="n">
+        <v>815.9299999999999</v>
+      </c>
+      <c r="C13" t="n">
+        <v>866.8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>874.23</v>
+      </c>
+      <c r="E13" t="n">
+        <v>870.515</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>11487.45 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" t="n">
+        <v>872.77</v>
+      </c>
+      <c r="C14" t="n">
+        <v>915.97</v>
+      </c>
+      <c r="D14" t="n">
+        <v>918.5700000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>917.27</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>10901.92 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" t="n">
+        <v>908.24</v>
+      </c>
+      <c r="C15" t="n">
+        <v>964.48</v>
+      </c>
+      <c r="D15" t="n">
+        <v>966.09</v>
+      </c>
+      <c r="E15" t="n">
+        <v>965.2850000000001</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10359.63 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="n">
+        <v>959.24</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1008.94</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1011.39</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1010.165</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>9899.37 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="n">
+        <v>999.8200000000001</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1054.38</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1053.21</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1053.795</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>9489.51 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1052.48</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1096.77</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1097.87</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1097.32</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>9113.11 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1076.21</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1125.28</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1126.64</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1125.96</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>8881.31 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1110.34</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1162.2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1164.06</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1163.13</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>8597.49 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1151.54</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1206.89</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1212.72</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1209.805</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>8265.79 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1177.67</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1234.23</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1240.29</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1237.26</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>8082.38 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1206.48</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1258.78</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1259.94</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1259.36</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>7940.54 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1234.02</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1287.32</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1293.89</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1290.605</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>7748.3 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1264.32</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1311.44</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1321.03</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1316.235</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>7597.43 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1280.02</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1338.58</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1341.27</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1339.925</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>7463.1 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1298.92</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1363.45</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1352.14</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1357.795</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>7364.88 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1322.18</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1392.74</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1393.22</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1392.98</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>7178.85 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="n">
+        <v>1347.96</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1405.56</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1407.33</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1406.445</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>7110.13 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1368.86</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1426.76</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1427.92</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1427.34</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>7006.04 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" t="n">
+        <v>1385.64</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1445.14</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1445.1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1445.12</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>6919.84 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" t="n">
+        <v>1395.92</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1456.82</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1457.21</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1457.015</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>6863.35 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1418.17</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1482.85</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1482.73</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1482.79</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>6744.04 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" t="n">
+        <v>1439.71</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1500.22</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1495.76</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1497.99</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>6675.61 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1450.71</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1513.46</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1515.73</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1514.595</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>6602.43 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1462.34</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1531.82</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1527.03</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1529.425</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>6538.4 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1422.36</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1537.52</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1534.8</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1536.16</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>6509.74 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" t="n">
+        <v>1497.9</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1559.68</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1561.59</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1560.635</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>6407.65 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1473.5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1577.45</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1580.4</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1578.925</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>6333.42 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1519.34</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1584.8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1588.47</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1586.635</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>6302.65 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1531.37</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1597.71</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1594.49</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1596.1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>6265.27 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="n">
+        <v>1546.66</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1611.65</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1611.46</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1611.555</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>6205.19 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="n">
+        <v>1555.66</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1619.02</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1624.21</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1621.615</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>6166.69 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="n">
+        <v>1572.92</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1641.14</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1638.8</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1639.97</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>6097.67 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1585.72</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1644.77</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1653.23</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1649</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>6064.28 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1590.18</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1655.88</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1658.35</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1657.115</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>6034.58 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1603.01</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1668.96</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1672.06</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1670.51</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>5986.2 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1619.07</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1670.88</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1675.29</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1673.085</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>5976.98 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1625.35</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1685.29</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1692.91</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1689.1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>5920.31 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1633.14</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1698.2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1695.52</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1696.86</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>5893.24 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1639.98</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1704.63</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1704.61</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1704.62</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>5866.41 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" t="n">
+        <v>1649.63</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1713.5</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1711.77</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1712.635</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>5838.96 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1658.77</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1721.42</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1722.02</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1721.72</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>5808.15 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1677.6</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1734.23</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1731.97</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1733.1</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>5770.01 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1674.92</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1737.88</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1742.38</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1740.13</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>5746.7 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" t="n">
+        <v>1686.74</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1748.47</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1748.05</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1748.26</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>5719.97 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1690.74</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1755.16</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1755.02</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1755.09</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>5697.71 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" t="n">
+        <v>1701.9</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1766.33</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1764.39</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1765.36</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>5664.57 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1707.76</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1772.93</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1782.99</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1777.96</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>5624.42 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" t="n">
+        <v>1721.96</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1786.33</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1788.2</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1787.265</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>5595.14 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" t="n">
+        <v>1725.79</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1790.14</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1790.69</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1790.415</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>5585.3 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" t="n">
+        <v>1720.42</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1793.45</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1795.82</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1794.635</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>5572.16 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1741.1</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1803.61</v>
+      </c>
+      <c r="D63" t="n">
+        <v>1800.37</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1801.99</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>5549.42 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" t="n">
+        <v>1742.85</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1810.09</v>
+      </c>
+      <c r="D64" t="n">
+        <v>1813.52</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1811.805</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>5519.36 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" t="n">
+        <v>1741.09</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1806.45</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1807.51</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1806.98</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>5534.1 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" t="n">
+        <v>1754.69</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1817.59</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1819.35</v>
+      </c>
+      <c r="E66" t="n">
+        <v>1818.47</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>5499.13 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" t="n">
+        <v>1761.93</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1823.79</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1822.72</v>
+      </c>
+      <c r="E67" t="n">
+        <v>1823.255</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>5484.7 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>65</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1764.78</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1829.95</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1828.46</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1829.205</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>5466.86 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1772.64</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1838.73</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1842.46</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1840.595</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>5433.03 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1778.81</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1848.01</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1844.48</v>
+      </c>
+      <c r="E70" t="n">
+        <v>1846.245</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>5416.4 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1769.17</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1843.38</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1844.47</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1843.925</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>5423.21 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>69</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1712.58</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1749.81</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1751.17</v>
+      </c>
+      <c r="E72" t="n">
+        <v>1750.49</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>5712.69 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>70</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1713.04</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1754.87</v>
+      </c>
+      <c r="D73" t="n">
+        <v>1758.82</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1756.845</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>5692.02 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1714.84</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1762.93</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1761.96</v>
+      </c>
+      <c r="E74" t="n">
+        <v>1762.445</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5673.94 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>72</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1729.17</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1767.13</v>
+      </c>
+      <c r="D75" t="n">
+        <v>1769.25</v>
+      </c>
+      <c r="E75" t="n">
+        <v>1768.19</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>5655.5 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>73</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1733.22</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1773.62</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1773.64</v>
+      </c>
+      <c r="E76" t="n">
+        <v>1773.63</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>5638.15 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>74</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1736.06</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1779.04</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1774.7</v>
+      </c>
+      <c r="E77" t="n">
+        <v>1776.87</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>5627.87 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>75</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1734.78</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1781.61</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1778.41</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1780.01</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>5617.95 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>76</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1746.22</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1786.62</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1784.64</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1785.63</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>5600.26 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>77</v>
+      </c>
+      <c r="B80" t="n">
+        <v>1745.15</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1792.58</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1790.37</v>
+      </c>
+      <c r="E80" t="n">
+        <v>1791.475</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>5581.99 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>78</v>
+      </c>
+      <c r="B81" t="n">
+        <v>1754.38</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1791.99</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1792.19</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1792.09</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>5580.08 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>79</v>
+      </c>
+      <c r="B82" t="n">
+        <v>1738.55</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1788.3</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1793.57</v>
+      </c>
+      <c r="E82" t="n">
+        <v>1790.935</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>5583.68 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>80</v>
+      </c>
+      <c r="B83" t="n">
+        <v>1760.83</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1800.53</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1800.22</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1800.375</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>5554.4 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>81</v>
+      </c>
+      <c r="B84" t="n">
+        <v>1762.88</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1798.62</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1802.2</v>
+      </c>
+      <c r="E84" t="n">
+        <v>1800.41</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>5554.29 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>82</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1756.22</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1799.48</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1802.67</v>
+      </c>
+      <c r="E85" t="n">
+        <v>1801.075</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>5552.24 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>83</v>
+      </c>
+      <c r="B86" t="n">
+        <v>1746.25</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1804.57</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1803.36</v>
+      </c>
+      <c r="E86" t="n">
+        <v>1803.965</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>5543.34 seconds</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>